<commit_message>
Fig. 5(d): mark the LightTools slice-11 hemisphere on the panel and in the workbook
Same series, same stack: LightTools p 0.2884, eta_ext 0.6595 / 0.8755, EQE
0.5550 / 0.8372 against the tracer's 0.2884, 0.6597 / 0.8755, 0.5551 / 0.8371
at AR = 1.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1WQ3WGcJw8tT3QK2n57xo
</commit_message>
<xml_diff>
--- a/sim/mla/mla_aspect_rawdata.xlsx
+++ b/sim/mla/mla_aspect_rawdata.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aspect sweep" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="flat reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alt shapes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_T vs angle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_R at AR=0.50" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LightTools slice 11" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_T vs angle" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B_R at AR=0.50" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -957,77 +958,105 @@
       <c r="A61" s="2" t="n"/>
       <c r="B61" t="inlineStr">
         <is>
-          <t>The numbers are for this generic stack; the shape of the curve is the message.</t>
+          <t>Every EQE is the matrix series of eq. (1); the closed form is not used.  At AR = 1 the tracer reproduces the</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>author's LightTools BSDF (sheet 'LightTools slice 11'), so the curve is on the same footing as Fig. 5(a),(b),(e).</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>The numbers are for this generic stack; the shape of the curve is the message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
         <is>
           <t>Sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  aspect sweep</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>what the panel plots: p, eta_ext and EQE against AR for both reflectors</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  flat reference</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>the lens-free interface, same stack</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  alt shapes</t>
+          <t xml:space="preserve">  aspect sweep</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>each lens family outside its own range (see above)</t>
+          <t>what the panel plots: p, eta_ext and EQE against AR for both reflectors</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  B_T vs angle</t>
+          <t xml:space="preserve">  flat reference</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>escape probability per 1-degree incidence bin, for every AR</t>
+          <t>the lens-free interface, same stack</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  alt shapes</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>each lens family outside its own range (see above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B_T vs angle</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>escape probability per 1-degree incidence bin, for every AR</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  B_R at AR=0.50</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>the full return matrix at the Ag optimum, rows = outgoing bin</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LightTools slice 11</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>the author's LightTools hemisphere BSDF (n_MLA 1.80) through the same series: p 0.2884, eta_ext 0.6595 (Al) / 0.8755 (Ag), EQE 0.5550 / 0.8372 - identical to the tracer's AR = 1.00 row to 3e-4, which is what validates the other aspect ratios</t>
         </is>
       </c>
     </row>
@@ -2305,6 +2334,80 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>reflector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>p_single_pass</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EQE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>0.288411</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>0.659498</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0.554953</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0.288411</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>0.875528</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.837167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11058,7 +11161,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>